<commit_message>
Update issuer financials spreadsheet
</commit_message>
<xml_diff>
--- a/data/issuer_financials.xlsx
+++ b/data/issuer_financials.xlsx
@@ -3126,58 +3126,52 @@
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ВУШ"</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>9717068640</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>Общество с ограниченной ответственностью "Специализированное Финансовое общество Совком Секьюр"</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>9703193909</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2025</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>10694433</v>
-      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
-        <v>-2549955</v>
+        <v>764758</v>
       </c>
       <c r="I43" t="n">
-        <v>213787</v>
+        <v>35192</v>
       </c>
       <c r="J43" t="n">
-        <v>330829</v>
+        <v>1286080</v>
       </c>
       <c r="K43" t="n">
-        <v>13895537</v>
+        <v>10632078</v>
       </c>
       <c r="L43" t="n">
-        <v>4607881</v>
+        <v>3400068</v>
       </c>
       <c r="M43" t="n">
-        <v>2583863</v>
+        <v>1853940</v>
       </c>
       <c r="N43" t="n">
-        <v>410758</v>
+        <v>764768</v>
       </c>
       <c r="O43" t="n">
-        <v>4971431</v>
+        <v>5356352</v>
       </c>
       <c r="P43" t="n">
-        <v>5382399</v>
+        <v>3590518</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/10703464</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12558868</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -3190,12 +3184,12 @@
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью «Специализированное финансовое общество СБ Секьютиризация»</t>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "БОРЕЦ КАПИТАЛ"</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>9704138298</t>
+          <t>9731098069</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3208,38 +3202,40 @@
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr"/>
+      <c r="F44" t="n">
+        <v>1023</v>
+      </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>-110007</v>
+        <v>5086</v>
       </c>
       <c r="I44" t="n">
-        <v>-2651331</v>
+        <v>-8655</v>
       </c>
       <c r="J44" t="n">
-        <v>465777</v>
+        <v>219</v>
       </c>
       <c r="K44" t="n">
-        <v>6436164</v>
+        <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>1374585</v>
+        <v>0</v>
       </c>
       <c r="M44" t="n">
-        <v>2595164</v>
+        <v>25</v>
       </c>
       <c r="N44" t="n">
-        <v>285806</v>
+        <v>223227</v>
       </c>
       <c r="O44" t="n">
-        <v>1960665</v>
+        <v>33333869</v>
       </c>
       <c r="P44" t="n">
-        <v>1374860</v>
+        <v>33311146</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/11849209</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/11927098</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -3252,56 +3248,54 @@
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ООО «СФО ВТБ РКС ЭТАЛОН»</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>9704147373</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>Общество с ограниченной ответственностью "ЛИЗИНГОВАЯ КОМПАНИЯ ПРОСТЫЕ РЕШЕНИЯ"</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>278181110</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2025</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
+      <c r="F45" t="n">
+        <v>2194489</v>
+      </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>6112293</v>
+        <v>155122</v>
       </c>
       <c r="I45" t="n">
-        <v>-9926195</v>
+        <v>-2086627</v>
       </c>
       <c r="J45" t="n">
-        <v>20467815</v>
+        <v>463109</v>
       </c>
       <c r="K45" t="n">
-        <v>144460215</v>
+        <v>11391448</v>
       </c>
       <c r="L45" t="n">
-        <v>31592025</v>
+        <v>3335362</v>
       </c>
       <c r="M45" t="n">
-        <v>10095850</v>
+        <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>9955602</v>
+        <v>1453344</v>
       </c>
       <c r="O45" t="n">
-        <v>62360167</v>
+        <v>5990866</v>
       </c>
       <c r="P45" t="n">
-        <v>35761493</v>
+        <v>3989488</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/11883254</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/508857</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -3314,18 +3308,14 @@
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью «Специализированное финансовое общество СБ Секьюритизация 2»</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>9704160303</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>Общество с ограниченной ответственностью «Специализированное финансовое общество СБ Секьютиризация»</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>9704138298</v>
+      </c>
+      <c r="D46" t="n">
+        <v>2025</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -3335,35 +3325,35 @@
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="n">
-        <v>406160</v>
+        <v>-110007</v>
       </c>
       <c r="I46" t="n">
-        <v>-1846540</v>
+        <v>-2651331</v>
       </c>
       <c r="J46" t="n">
-        <v>788495</v>
+        <v>465777</v>
       </c>
       <c r="K46" t="n">
-        <v>10097440</v>
+        <v>6436164</v>
       </c>
       <c r="L46" t="n">
-        <v>1629792</v>
+        <v>1374585</v>
       </c>
       <c r="M46" t="n">
-        <v>1867484</v>
+        <v>2595164</v>
       </c>
       <c r="N46" t="n">
-        <v>406093</v>
+        <v>285806</v>
       </c>
       <c r="O46" t="n">
-        <v>2587855</v>
+        <v>1960665</v>
       </c>
       <c r="P46" t="n">
-        <v>1629933</v>
+        <v>1374860</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/11930756</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/11849209</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -5154,58 +5144,52 @@
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "ГЛОРАКС"</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>9729387137</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>Общество с ограниченной ответственностью "Специализированное Финансовое общество Тб-4"</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>9703211185</v>
+      </c>
+      <c r="D75" t="n">
+        <v>2025</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F75" t="n">
-        <v>3057693</v>
-      </c>
+      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="n">
-        <v>352891</v>
+        <v>977720</v>
       </c>
       <c r="I75" t="n">
-        <v>-2487508</v>
+        <v>-1274588</v>
       </c>
       <c r="J75" t="n">
-        <v>17468</v>
+        <v>2631244</v>
       </c>
       <c r="K75" t="n">
-        <v>15888211</v>
+        <v>20526472</v>
       </c>
       <c r="L75" t="n">
-        <v>7131352</v>
+        <v>4223028</v>
       </c>
       <c r="M75" t="n">
-        <v>3563226</v>
+        <v>1495620</v>
       </c>
       <c r="N75" t="n">
-        <v>5262202</v>
+        <v>977730</v>
       </c>
       <c r="O75" t="n">
-        <v>9887498</v>
+        <v>7130263</v>
       </c>
       <c r="P75" t="n">
-        <v>7607515</v>
+        <v>4225049</v>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12558009</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12680884</t>
         </is>
       </c>
       <c r="R75" t="inlineStr">
@@ -5218,58 +5202,52 @@
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "ГРУППА ПОЗИТИВ"</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>9718077239</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>Общество с ограниченной ответственностью "Специализированное Финансовое общество Сплит Финанс"</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>9703209122</v>
+      </c>
+      <c r="D76" t="n">
+        <v>2025</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F76" t="n">
-        <v>0</v>
-      </c>
+      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="n">
-        <v>-2319012</v>
+        <v>832800</v>
       </c>
       <c r="I76" t="n">
-        <v>-3043148</v>
+        <v>-627668</v>
       </c>
       <c r="J76" t="n">
-        <v>85073</v>
+        <v>3157507</v>
       </c>
       <c r="K76" t="n">
-        <v>20333431</v>
+        <v>12321587</v>
       </c>
       <c r="L76" t="n">
-        <v>533431</v>
+        <v>4622403</v>
       </c>
       <c r="M76" t="n">
-        <v>3093490</v>
+        <v>794736</v>
       </c>
       <c r="N76" t="n">
-        <v>14618010</v>
+        <v>832810</v>
       </c>
       <c r="O76" t="n">
-        <v>6251325</v>
+        <v>10288657</v>
       </c>
       <c r="P76" t="n">
-        <v>542917</v>
+        <v>4649009</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/10388722</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12663922</t>
         </is>
       </c>
       <c r="R76" t="inlineStr">
@@ -5282,58 +5260,52 @@
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "КАРШЕРИНГ РУССИЯ"</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>9718236471</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>Общество с ограниченной ответственностью "Специализированное Финансовое общество Тб-6"</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>9703221553</v>
+      </c>
+      <c r="D77" t="n">
+        <v>2025</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F77" t="n">
-        <v>26088727</v>
-      </c>
+      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
-        <v>-3628694</v>
+        <v>421691</v>
       </c>
       <c r="I77" t="n">
-        <v>6086337</v>
+        <v>-16243</v>
       </c>
       <c r="J77" t="n">
-        <v>1230217</v>
+        <v>1996969</v>
       </c>
       <c r="K77" t="n">
-        <v>18535372</v>
+        <v>31400566</v>
       </c>
       <c r="L77" t="n">
-        <v>10535372</v>
+        <v>191416</v>
       </c>
       <c r="M77" t="n">
-        <v>5647179</v>
+        <v>191760</v>
       </c>
       <c r="N77" t="n">
-        <v>6060673</v>
+        <v>421701</v>
       </c>
       <c r="O77" t="n">
-        <v>6682880</v>
+        <v>11406621</v>
       </c>
       <c r="P77" t="n">
-        <v>17515458</v>
+        <v>592089</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12289607</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12744848</t>
         </is>
       </c>
       <c r="R77" t="inlineStr">
@@ -5346,12 +5318,12 @@
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "ФАБРИКА ПО"</t>
+          <t>Общество с ограниченной ответственностью "Профессиональная коллекторская организация "Агентство судебного взыскания"</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>9726092897</t>
+          <t>7841019595</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5364,38 +5336,40 @@
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
+      <c r="F78" t="n">
+        <v>2813950</v>
+      </c>
       <c r="G78" t="inlineStr"/>
       <c r="H78" t="n">
-        <v>26111</v>
+        <v>289449</v>
       </c>
       <c r="I78" t="n">
-        <v>-116300</v>
+        <v>-782507</v>
       </c>
       <c r="J78" t="n">
-        <v>58920</v>
+        <v>439421</v>
       </c>
       <c r="K78" t="n">
-        <v>2012480</v>
+        <v>3335265</v>
       </c>
       <c r="L78" t="n">
-        <v>1961794</v>
+        <v>1661751</v>
       </c>
       <c r="M78" t="n">
-        <v>94487</v>
+        <v>634394</v>
       </c>
       <c r="N78" t="n">
-        <v>15655004</v>
+        <v>718092</v>
       </c>
       <c r="O78" t="n">
-        <v>3749182</v>
+        <v>4036728</v>
       </c>
       <c r="P78" t="n">
-        <v>3460790</v>
+        <v>1804336</v>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12624794</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/9111808</t>
         </is>
       </c>
       <c r="R78" t="inlineStr">
@@ -5408,12 +5382,12 @@
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "Профессиональная коллекторская организация "Агентство судебного взыскания"</t>
+          <t>Общество с ограниченной ответственностью "ЛЕГЕНДА"</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>7841019595</t>
+          <t>7840438730</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5427,39 +5401,39 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>2813950</v>
+        <v>2574338</v>
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="n">
-        <v>289449</v>
+        <v>676819</v>
       </c>
       <c r="I79" t="n">
-        <v>-782507</v>
+        <v>1424991</v>
       </c>
       <c r="J79" t="n">
-        <v>439421</v>
+        <v>2369150</v>
       </c>
       <c r="K79" t="n">
-        <v>3335265</v>
+        <v>13269288</v>
       </c>
       <c r="L79" t="n">
-        <v>1661751</v>
+        <v>5143359</v>
       </c>
       <c r="M79" t="n">
-        <v>634394</v>
+        <v>1792096</v>
       </c>
       <c r="N79" t="n">
-        <v>718092</v>
+        <v>988224</v>
       </c>
       <c r="O79" t="n">
-        <v>4036728</v>
+        <v>7760068</v>
       </c>
       <c r="P79" t="n">
-        <v>1804336</v>
+        <v>5682975</v>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/9111808</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/122728</t>
         </is>
       </c>
       <c r="R79" t="inlineStr">
@@ -5472,12 +5446,12 @@
       <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ЛЕГЕНДА"</t>
+          <t>Общество с ограниченной ответственностью Профессиональная коллекторская организация "Филберт"</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>7840438730</t>
+          <t>7841430420</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5491,39 +5465,39 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>2574338</v>
+        <v>8586868</v>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="n">
-        <v>676819</v>
+        <v>3152859</v>
       </c>
       <c r="I80" t="n">
-        <v>1424991</v>
+        <v>-2961381</v>
       </c>
       <c r="J80" t="n">
-        <v>2369150</v>
+        <v>130669</v>
       </c>
       <c r="K80" t="n">
-        <v>13269288</v>
+        <v>4275711</v>
       </c>
       <c r="L80" t="n">
-        <v>5143359</v>
+        <v>2275535</v>
       </c>
       <c r="M80" t="n">
-        <v>1792096</v>
+        <v>560901</v>
       </c>
       <c r="N80" t="n">
-        <v>988224</v>
+        <v>9134906</v>
       </c>
       <c r="O80" t="n">
-        <v>7760068</v>
+        <v>13555399</v>
       </c>
       <c r="P80" t="n">
-        <v>5682975</v>
+        <v>2486647</v>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/122728</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/1655225</t>
         </is>
       </c>
       <c r="R80" t="inlineStr">
@@ -5536,12 +5510,12 @@
       <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью Профессиональная коллекторская организация "Филберт"</t>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "МВ ФИНАНС"</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>7841430420</t>
+          <t>9701168311</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -5554,40 +5528,38 @@
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F81" t="n">
-        <v>8586868</v>
-      </c>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="n">
-        <v>3152859</v>
+        <v>3493</v>
       </c>
       <c r="I81" t="n">
-        <v>-2961381</v>
+        <v>-2391603</v>
       </c>
       <c r="J81" t="n">
-        <v>130669</v>
+        <v>44911</v>
       </c>
       <c r="K81" t="n">
-        <v>4275711</v>
+        <v>7725451</v>
       </c>
       <c r="L81" t="n">
-        <v>2275535</v>
+        <v>5759320</v>
       </c>
       <c r="M81" t="n">
-        <v>560901</v>
+        <v>2261066</v>
       </c>
       <c r="N81" t="n">
-        <v>9134906</v>
+        <v>95811</v>
       </c>
       <c r="O81" t="n">
-        <v>13555399</v>
+        <v>5828974</v>
       </c>
       <c r="P81" t="n">
-        <v>2486647</v>
+        <v>5765046</v>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/1655225</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/11476959</t>
         </is>
       </c>
       <c r="R81" t="inlineStr">
@@ -5600,12 +5572,12 @@
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "МВ ФИНАНС"</t>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "ВУШ"</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>9701168311</t>
+          <t>9717068640</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5618,38 +5590,40 @@
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
+      <c r="F82" t="n">
+        <v>10694433</v>
+      </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
-        <v>3493</v>
+        <v>-2549955</v>
       </c>
       <c r="I82" t="n">
-        <v>-2391603</v>
+        <v>213787</v>
       </c>
       <c r="J82" t="n">
-        <v>44911</v>
+        <v>330829</v>
       </c>
       <c r="K82" t="n">
-        <v>7725451</v>
+        <v>13895537</v>
       </c>
       <c r="L82" t="n">
-        <v>5759320</v>
+        <v>4607881</v>
       </c>
       <c r="M82" t="n">
-        <v>2261066</v>
+        <v>2583863</v>
       </c>
       <c r="N82" t="n">
-        <v>95811</v>
+        <v>410758</v>
       </c>
       <c r="O82" t="n">
-        <v>5828974</v>
+        <v>4971431</v>
       </c>
       <c r="P82" t="n">
-        <v>5765046</v>
+        <v>5382399</v>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/11476959</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/10703464</t>
         </is>
       </c>
       <c r="R82" t="inlineStr">
@@ -5662,12 +5636,12 @@
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "Специализированное финансовое общество ТБ-5"</t>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО ГРУППА КОМПАНИЙ "СЕГЕЖА"</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>9703206788</t>
+          <t>9703024202</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5680,38 +5654,40 @@
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
+      <c r="F83" t="n">
+        <v>3234274</v>
+      </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
-        <v>627562</v>
+        <v>-81659202</v>
       </c>
       <c r="I83" t="n">
-        <v>2054</v>
+        <v>-15560254</v>
       </c>
       <c r="J83" t="n">
-        <v>2567719</v>
+        <v>2171160</v>
       </c>
       <c r="K83" t="n">
-        <v>16587377</v>
+        <v>68989930</v>
       </c>
       <c r="L83" t="n">
-        <v>336877</v>
+        <v>28619951</v>
       </c>
       <c r="M83" t="n">
-        <v>337763</v>
+        <v>17966508</v>
       </c>
       <c r="N83" t="n">
-        <v>627572</v>
+        <v>69901335</v>
       </c>
       <c r="O83" t="n">
-        <v>6522558</v>
+        <v>16693441</v>
       </c>
       <c r="P83" t="n">
-        <v>636777</v>
+        <v>29540756</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12646488</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/11477936</t>
         </is>
       </c>
       <c r="R83" t="inlineStr">
@@ -5724,12 +5700,12 @@
       <c r="A84" t="inlineStr"/>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО ГРУППА КОМПАНИЙ "СЕГЕЖА"</t>
+          <t>ООО «БИННОФАРМ ГРУПП»</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>9703024202</t>
+          <t>9704005675</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -5743,39 +5719,39 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>3234274</v>
+        <v>39152023</v>
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
-        <v>-81659202</v>
+        <v>-3437553</v>
       </c>
       <c r="I84" t="n">
-        <v>-15560254</v>
+        <v>-10088180</v>
       </c>
       <c r="J84" t="n">
-        <v>2171160</v>
+        <v>2741369</v>
       </c>
       <c r="K84" t="n">
-        <v>68989930</v>
+        <v>31048484</v>
       </c>
       <c r="L84" t="n">
-        <v>28619951</v>
+        <v>27198484</v>
       </c>
       <c r="M84" t="n">
-        <v>17966508</v>
+        <v>6612689</v>
       </c>
       <c r="N84" t="n">
-        <v>69901335</v>
+        <v>28187621</v>
       </c>
       <c r="O84" t="n">
-        <v>16693441</v>
+        <v>49838344</v>
       </c>
       <c r="P84" t="n">
-        <v>29540756</v>
+        <v>65495561</v>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/11477936</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/11181494</t>
         </is>
       </c>
       <c r="R84" t="inlineStr">
@@ -5788,12 +5764,12 @@
       <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "СПЕЦИАЛИЗИРОВАННОЕ ФИНАНСОВОЕ ОБЩЕСТВО "СБ СЕКЬЮРИТИЗАЦИЯ 5"</t>
+          <t>Публичное Акционерное общество "Лизинговая компания "Европлан"</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>9703163693</t>
+          <t>9705101614</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -5806,32 +5782,40 @@
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr"/>
+      <c r="F85" t="n">
+        <v>59966125</v>
+      </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
-        <v>-65</v>
+        <v>4034508</v>
       </c>
       <c r="I85" t="n">
-        <v>-266</v>
+        <v>84799387</v>
       </c>
       <c r="J85" t="n">
-        <v>13</v>
-      </c>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr"/>
+        <v>7477939</v>
+      </c>
+      <c r="K85" t="n">
+        <v>136124027</v>
+      </c>
+      <c r="L85" t="n">
+        <v>73233527</v>
+      </c>
+      <c r="M85" t="n">
+        <v>35514645</v>
+      </c>
       <c r="N85" t="n">
-        <v>13</v>
+        <v>36127674</v>
       </c>
       <c r="O85" t="n">
-        <v>13</v>
+        <v>113385304</v>
       </c>
       <c r="P85" t="n">
-        <v>0</v>
+        <v>85482683</v>
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12333197</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/10283154</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
@@ -5844,12 +5828,12 @@
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "Специализированное Финансовое общество Совком Секьюр"</t>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "КАРШЕРИНГ РУССИЯ"</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>9703193909</t>
+          <t>9718236471</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5862,38 +5846,40 @@
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr"/>
+      <c r="F86" t="n">
+        <v>26088727</v>
+      </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="n">
-        <v>764758</v>
+        <v>-3628694</v>
       </c>
       <c r="I86" t="n">
-        <v>35192</v>
+        <v>6086337</v>
       </c>
       <c r="J86" t="n">
-        <v>1286080</v>
+        <v>1230217</v>
       </c>
       <c r="K86" t="n">
-        <v>10632078</v>
+        <v>18535372</v>
       </c>
       <c r="L86" t="n">
-        <v>3400068</v>
+        <v>10535372</v>
       </c>
       <c r="M86" t="n">
-        <v>1853940</v>
+        <v>5647179</v>
       </c>
       <c r="N86" t="n">
-        <v>764768</v>
+        <v>6060673</v>
       </c>
       <c r="O86" t="n">
-        <v>5356352</v>
+        <v>6682880</v>
       </c>
       <c r="P86" t="n">
-        <v>3590518</v>
+        <v>17515458</v>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12558868</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12289607</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -5906,12 +5892,12 @@
       <c r="A87" t="inlineStr"/>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "Специализированное Финансовое общество Тб-4"</t>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "ГРУППА ПОЗИТИВ"</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>9703211185</t>
+          <t>9718077239</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5924,38 +5910,40 @@
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr"/>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
-        <v>977720</v>
+        <v>-2319012</v>
       </c>
       <c r="I87" t="n">
-        <v>-1274588</v>
+        <v>-3043148</v>
       </c>
       <c r="J87" t="n">
-        <v>2631244</v>
+        <v>85073</v>
       </c>
       <c r="K87" t="n">
-        <v>20526472</v>
+        <v>20333431</v>
       </c>
       <c r="L87" t="n">
-        <v>4223028</v>
+        <v>533431</v>
       </c>
       <c r="M87" t="n">
-        <v>1495620</v>
+        <v>3093490</v>
       </c>
       <c r="N87" t="n">
-        <v>977730</v>
+        <v>14618010</v>
       </c>
       <c r="O87" t="n">
-        <v>7130263</v>
+        <v>6251325</v>
       </c>
       <c r="P87" t="n">
-        <v>4225049</v>
+        <v>542917</v>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12680884</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/10388722</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -5968,12 +5956,12 @@
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "Специализированное Финансовое общество Сплит Финанс"</t>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "ФАБРИКА ПО"</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>9703209122</t>
+          <t>9726092897</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5989,35 +5977,35 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
-        <v>832800</v>
+        <v>26111</v>
       </c>
       <c r="I88" t="n">
-        <v>-627668</v>
+        <v>-116300</v>
       </c>
       <c r="J88" t="n">
-        <v>3157507</v>
+        <v>58920</v>
       </c>
       <c r="K88" t="n">
-        <v>12321587</v>
+        <v>2012480</v>
       </c>
       <c r="L88" t="n">
-        <v>4622403</v>
+        <v>1961794</v>
       </c>
       <c r="M88" t="n">
-        <v>794736</v>
+        <v>94487</v>
       </c>
       <c r="N88" t="n">
-        <v>832810</v>
+        <v>15655004</v>
       </c>
       <c r="O88" t="n">
-        <v>10288657</v>
+        <v>3749182</v>
       </c>
       <c r="P88" t="n">
-        <v>4649009</v>
+        <v>3460790</v>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12663922</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12624794</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -6030,12 +6018,12 @@
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "Специализированное Финансовое общество Тб-6"</t>
+          <t>ПУБЛИЧНОЕ АКЦИОНЕРНОЕ ОБЩЕСТВО "ГЛОРАКС"</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>9703221553</t>
+          <t>9729387137</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -6048,38 +6036,40 @@
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr"/>
+      <c r="F89" t="n">
+        <v>3057693</v>
+      </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
-        <v>421691</v>
+        <v>352891</v>
       </c>
       <c r="I89" t="n">
-        <v>-16243</v>
+        <v>-2487508</v>
       </c>
       <c r="J89" t="n">
-        <v>1996969</v>
+        <v>17468</v>
       </c>
       <c r="K89" t="n">
-        <v>31400566</v>
+        <v>15888211</v>
       </c>
       <c r="L89" t="n">
-        <v>191416</v>
+        <v>7131352</v>
       </c>
       <c r="M89" t="n">
-        <v>191760</v>
+        <v>3563226</v>
       </c>
       <c r="N89" t="n">
-        <v>421701</v>
+        <v>5262202</v>
       </c>
       <c r="O89" t="n">
-        <v>11406621</v>
+        <v>9887498</v>
       </c>
       <c r="P89" t="n">
-        <v>592089</v>
+        <v>7607515</v>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12744848</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12558009</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -6092,58 +6082,52 @@
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr">
         <is>
-          <t>ООО «БИННОФАРМ ГРУПП»</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>9704005675</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "СПЕЦИАЛИЗИРОВАННОЕ ФИНАНСОВОЕ ОБЩЕСТВО СБ СЕКЬЮРИТИЗАЦИЯ 3"</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>9704262880</v>
+      </c>
+      <c r="D90" t="n">
+        <v>2025</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F90" t="n">
-        <v>39152023</v>
-      </c>
+      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
-        <v>-3437553</v>
+        <v>867964</v>
       </c>
       <c r="I90" t="n">
-        <v>-10088180</v>
+        <v>-10844</v>
       </c>
       <c r="J90" t="n">
-        <v>2741369</v>
+        <v>1901818</v>
       </c>
       <c r="K90" t="n">
-        <v>31048484</v>
+        <v>22434769</v>
       </c>
       <c r="L90" t="n">
-        <v>27198484</v>
+        <v>2918653</v>
       </c>
       <c r="M90" t="n">
-        <v>6612689</v>
+        <v>268761</v>
       </c>
       <c r="N90" t="n">
-        <v>28187621</v>
+        <v>867973</v>
       </c>
       <c r="O90" t="n">
-        <v>49838344</v>
+        <v>5010242</v>
       </c>
       <c r="P90" t="n">
-        <v>65495561</v>
+        <v>2921170</v>
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/11181494</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12724282</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -6156,11 +6140,11 @@
       <c r="A91" t="inlineStr"/>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Общество с ограниченной ответственностью "ЛИЗИНГОВАЯ КОМПАНИЯ ПРОСТЫЕ РЕШЕНИЯ"</t>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "СПЕЦИАЛИЗИРОВАННОЕ ФИНАНСОВОЕ ОБЩЕСТВО АЛЬФА ФАБРИКА ПК-1"</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>278181110</v>
+        <v>9704256936</v>
       </c>
       <c r="D91" t="n">
         <v>2025</v>
@@ -6170,40 +6154,38 @@
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F91" t="n">
-        <v>2194489</v>
-      </c>
+      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
-        <v>155122</v>
+        <v>462857</v>
       </c>
       <c r="I91" t="n">
-        <v>-2086627</v>
+        <v>-690900</v>
       </c>
       <c r="J91" t="n">
-        <v>463109</v>
+        <v>1467792</v>
       </c>
       <c r="K91" t="n">
-        <v>11391448</v>
+        <v>12652034</v>
       </c>
       <c r="L91" t="n">
-        <v>3335362</v>
+        <v>2707767</v>
       </c>
       <c r="M91" t="n">
-        <v>0</v>
+        <v>740205</v>
       </c>
       <c r="N91" t="n">
-        <v>1453344</v>
+        <v>462867</v>
       </c>
       <c r="O91" t="n">
-        <v>5990866</v>
+        <v>4761718</v>
       </c>
       <c r="P91" t="n">
-        <v>3989488</v>
+        <v>2710789</v>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/508857</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12624837</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -6216,58 +6198,52 @@
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "БОРЕЦ КАПИТАЛ"</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>9731098069</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "СПЕЦИАЛИЗИРОВАННОЕ ФИНАНСОВОЕ ОБЩЕСТВО АЛЬФА ФАБРИКА ПК-2"</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>9704264662</v>
+      </c>
+      <c r="D92" t="n">
+        <v>2025</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F92" t="n">
-        <v>1023</v>
-      </c>
+      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="n">
-        <v>5086</v>
+        <v>966</v>
       </c>
       <c r="I92" t="n">
-        <v>-8655</v>
+        <v>-439</v>
       </c>
       <c r="J92" t="n">
-        <v>219</v>
+        <v>2571</v>
       </c>
       <c r="K92" t="n">
-        <v>0</v>
+        <v>3133</v>
       </c>
       <c r="L92" t="n">
-        <v>0</v>
+        <v>3133</v>
       </c>
       <c r="M92" t="n">
-        <v>25</v>
+        <v>133</v>
       </c>
       <c r="N92" t="n">
-        <v>223227</v>
+        <v>-956</v>
       </c>
       <c r="O92" t="n">
-        <v>33333869</v>
+        <v>2571</v>
       </c>
       <c r="P92" t="n">
-        <v>33311146</v>
+        <v>3527</v>
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/11927098</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12755483</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -6280,58 +6256,46 @@
       <c r="A93" t="inlineStr"/>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Публичное Акционерное общество "Лизинговая компания "Европлан"</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>9705101614</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>Общество с ограниченной ответственностью "СПЕЦИАЛИЗИРОВАННОЕ ФИНАНСОВОЕ ОБЩЕСТВО "СБ СЕКЬЮРИТИЗАЦИЯ 5"</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>9703163693</v>
+      </c>
+      <c r="D93" t="n">
+        <v>2025</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
           <t>тыс. руб.</t>
         </is>
       </c>
-      <c r="F93" t="n">
-        <v>59966125</v>
-      </c>
+      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="n">
-        <v>4034508</v>
+        <v>-65</v>
       </c>
       <c r="I93" t="n">
-        <v>84799387</v>
+        <v>-266</v>
       </c>
       <c r="J93" t="n">
-        <v>7477939</v>
-      </c>
-      <c r="K93" t="n">
-        <v>136124027</v>
-      </c>
-      <c r="L93" t="n">
-        <v>73233527</v>
-      </c>
-      <c r="M93" t="n">
-        <v>35514645</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
       <c r="N93" t="n">
-        <v>36127674</v>
+        <v>13</v>
       </c>
       <c r="O93" t="n">
-        <v>113385304</v>
+        <v>13</v>
       </c>
       <c r="P93" t="n">
-        <v>85482683</v>
+        <v>0</v>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/10283154</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12333197</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -6344,18 +6308,14 @@
       <c r="A94" t="inlineStr"/>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "СПЕЦИАЛИЗИРОВАННОЕ ФИНАНСОВОЕ ОБЩЕСТВО АЛЬФА ФАБРИКА ПК-1"</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>9704256936</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>ООО «СФО ВТБ РКС ЭТАЛОН»</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>9704147373</v>
+      </c>
+      <c r="D94" t="n">
+        <v>2025</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -6365,35 +6325,35 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="n">
-        <v>462857</v>
+        <v>6112293</v>
       </c>
       <c r="I94" t="n">
-        <v>-690900</v>
+        <v>-9926195</v>
       </c>
       <c r="J94" t="n">
-        <v>1467792</v>
+        <v>20467815</v>
       </c>
       <c r="K94" t="n">
-        <v>12652034</v>
+        <v>144460215</v>
       </c>
       <c r="L94" t="n">
-        <v>2707767</v>
+        <v>31592025</v>
       </c>
       <c r="M94" t="n">
-        <v>740205</v>
+        <v>10095850</v>
       </c>
       <c r="N94" t="n">
-        <v>462867</v>
+        <v>9955602</v>
       </c>
       <c r="O94" t="n">
-        <v>4761718</v>
+        <v>62360167</v>
       </c>
       <c r="P94" t="n">
-        <v>2710789</v>
+        <v>35761493</v>
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12624837</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/11883254</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -6406,18 +6366,14 @@
       <c r="A95" t="inlineStr"/>
       <c r="B95" t="inlineStr">
         <is>
-          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "СПЕЦИАЛИЗИРОВАННОЕ ФИНАНСОВОЕ ОБЩЕСТВО СБ СЕКЬЮРИТИЗАЦИЯ 3"</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>9704262880</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>Общество с ограниченной ответственностью «Специализированное финансовое общество СБ Секьюритизация 2»</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>9704160303</v>
+      </c>
+      <c r="D95" t="n">
+        <v>2025</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -6427,35 +6383,35 @@
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="n">
-        <v>867964</v>
+        <v>406160</v>
       </c>
       <c r="I95" t="n">
-        <v>-10844</v>
+        <v>-1846540</v>
       </c>
       <c r="J95" t="n">
-        <v>1901818</v>
+        <v>788495</v>
       </c>
       <c r="K95" t="n">
-        <v>22434769</v>
+        <v>10097440</v>
       </c>
       <c r="L95" t="n">
-        <v>2918653</v>
+        <v>1629792</v>
       </c>
       <c r="M95" t="n">
-        <v>268761</v>
+        <v>1867484</v>
       </c>
       <c r="N95" t="n">
-        <v>867973</v>
+        <v>406093</v>
       </c>
       <c r="O95" t="n">
-        <v>5010242</v>
+        <v>2587855</v>
       </c>
       <c r="P95" t="n">
-        <v>2921170</v>
+        <v>1629933</v>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12724282</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/11930756</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -6468,18 +6424,14 @@
       <c r="A96" t="inlineStr"/>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ОБЩЕСТВО С ОГРАНИЧЕННОЙ ОТВЕТСТВЕННОСТЬЮ "СПЕЦИАЛИЗИРОВАННОЕ ФИНАНСОВОЕ ОБЩЕСТВО АЛЬФА ФАБРИКА ПК-2"</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>9704264662</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
+          <t>Общество с ограниченной ответственностью "Специализированное финансовое общество ТБ-5"</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>9703206788</v>
+      </c>
+      <c r="D96" t="n">
+        <v>2025</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -6489,35 +6441,35 @@
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="n">
-        <v>966</v>
+        <v>627562</v>
       </c>
       <c r="I96" t="n">
-        <v>-439</v>
+        <v>2054</v>
       </c>
       <c r="J96" t="n">
-        <v>2571</v>
+        <v>2567719</v>
       </c>
       <c r="K96" t="n">
-        <v>3133</v>
+        <v>16587377</v>
       </c>
       <c r="L96" t="n">
-        <v>3133</v>
+        <v>336877</v>
       </c>
       <c r="M96" t="n">
-        <v>133</v>
+        <v>337763</v>
       </c>
       <c r="N96" t="n">
-        <v>-956</v>
+        <v>627572</v>
       </c>
       <c r="O96" t="n">
-        <v>2571</v>
+        <v>6522558</v>
       </c>
       <c r="P96" t="n">
-        <v>3527</v>
+        <v>636777</v>
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>https://bo.nalog.gov.ru/organizations-card/12755483</t>
+          <t>https://bo.nalog.gov.ru/organizations-card/12646488</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">

</xml_diff>